<commit_message>
Fix Q3/Q4 target display, restore H2 target, add sidebar sticky positioning, add Q2 pipeline and business plan data, fix unused import build error
</commit_message>
<xml_diff>
--- a/files/Opportunity Pipeline Q1.xlsx
+++ b/files/Opportunity Pipeline Q1.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30306"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30305"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://techpayai-my.sharepoint.com/personal/dilip_s_techpay_ai/Documents/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="226" documentId="8_{B9D4CF75-84DE-4256-A0DF-80742AC4FA1C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{C5A679B8-0128-4A5B-89D6-A61B749BC19B}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{D0E2F4E8-99C1-4647-89CF-6DB617A91F2B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{C2124116-525B-40F1-AC9B-01E56399BFA6}"/>
   </bookViews>
@@ -6590,7 +6590,15 @@
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{B06AE79E-9194-4B59-B9CC-9B6E72DFA18C}" name="PipelineData" displayName="PipelineData" ref="A1:Z380" totalsRowShown="0">
-  <autoFilter ref="A1:Z380" xr:uid="{B06AE79E-9194-4B59-B9CC-9B6E72DFA18C}"/>
+  <autoFilter ref="A1:Z380" xr:uid="{B06AE79E-9194-4B59-B9CC-9B6E72DFA18C}">
+    <filterColumn colId="5">
+      <filters>
+        <filter val="Ajay Patodia"/>
+        <filter val="Hrushikesh Bagade"/>
+        <filter val="Yusufali Petiwala"/>
+      </filters>
+    </filterColumn>
+  </autoFilter>
   <tableColumns count="26">
     <tableColumn id="1" xr3:uid="{DCA610E8-1315-4324-B57D-7FB2A163A990}" name="Created Time"/>
     <tableColumn id="2" xr3:uid="{729FC86D-7420-4183-BE52-156A46C8048B}" name="Opportunity Number"/>
@@ -6941,33 +6949,10 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F355E0A6-1A35-4BEA-977E-E5FE8304A0F7}">
   <dimension ref="A1:Z380"/>
-  <sheetFormatPr defaultRowHeight="14.45"/>
+  <sheetFormatPr defaultColWidth="11.28515625" defaultRowHeight="14.45"/>
   <cols>
-    <col min="1" max="1" width="19.85546875" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="21.85546875" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="56.7109375" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="24.5703125" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="70.42578125" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="20.42578125" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="70.42578125" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="18.7109375" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="15.42578125" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="18.140625" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="25.85546875" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="23.42578125" bestFit="1" customWidth="1"/>
-    <col min="13" max="14" width="13.7109375" bestFit="1" customWidth="1"/>
-    <col min="15" max="15" width="14.85546875" style="6" bestFit="1" customWidth="1"/>
-    <col min="16" max="16" width="23" bestFit="1" customWidth="1"/>
-    <col min="17" max="17" width="20.7109375" bestFit="1" customWidth="1"/>
-    <col min="18" max="18" width="22" bestFit="1" customWidth="1"/>
-    <col min="19" max="19" width="16" bestFit="1" customWidth="1"/>
-    <col min="20" max="20" width="13" bestFit="1" customWidth="1"/>
-    <col min="21" max="21" width="13.7109375" bestFit="1" customWidth="1"/>
-    <col min="22" max="22" width="22" bestFit="1" customWidth="1"/>
-    <col min="23" max="23" width="13.5703125" bestFit="1" customWidth="1"/>
-    <col min="24" max="24" width="18" bestFit="1" customWidth="1"/>
-    <col min="25" max="25" width="174.85546875" bestFit="1" customWidth="1"/>
-    <col min="26" max="26" width="18.140625" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="12.5703125" style="6" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:26" ht="15">
@@ -7050,7 +7035,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="2" spans="1:26" ht="15">
+    <row r="2" spans="1:26" ht="15" hidden="1">
       <c r="A2" s="1">
         <v>46177.646527777775</v>
       </c>
@@ -7130,7 +7115,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="3" spans="1:26" ht="15">
+    <row r="3" spans="1:26" ht="15" hidden="1">
       <c r="A3" s="1">
         <v>46208.540972222225</v>
       </c>
@@ -7210,7 +7195,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="4" spans="1:26" ht="15">
+    <row r="4" spans="1:26" ht="15" hidden="1">
       <c r="A4" s="1">
         <v>46331.740277777775</v>
       </c>
@@ -9530,7 +9515,7 @@
         <v>68</v>
       </c>
     </row>
-    <row r="33" spans="1:26" ht="15">
+    <row r="33" spans="1:26" ht="15" hidden="1">
       <c r="A33" t="s">
         <v>207</v>
       </c>
@@ -9610,7 +9595,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="34" spans="1:26" ht="15">
+    <row r="34" spans="1:26" ht="15" hidden="1">
       <c r="A34" t="s">
         <v>214</v>
       </c>
@@ -9690,7 +9675,7 @@
         <v>225</v>
       </c>
     </row>
-    <row r="35" spans="1:26" ht="15">
+    <row r="35" spans="1:26" ht="15" hidden="1">
       <c r="A35" s="1">
         <v>46270.557638888888</v>
       </c>
@@ -9770,7 +9755,7 @@
         <v>225</v>
       </c>
     </row>
-    <row r="36" spans="1:26" ht="15">
+    <row r="36" spans="1:26" ht="15" hidden="1">
       <c r="A36" t="s">
         <v>231</v>
       </c>
@@ -9850,7 +9835,7 @@
         <v>225</v>
       </c>
     </row>
-    <row r="37" spans="1:26" ht="15">
+    <row r="37" spans="1:26" ht="15" hidden="1">
       <c r="A37" s="1">
         <v>46177.511111111111</v>
       </c>
@@ -9930,7 +9915,7 @@
         <v>246</v>
       </c>
     </row>
-    <row r="38" spans="1:26" ht="15">
+    <row r="38" spans="1:26" ht="15" hidden="1">
       <c r="A38" t="s">
         <v>247</v>
       </c>
@@ -10010,7 +9995,7 @@
         <v>32</v>
       </c>
     </row>
-    <row r="39" spans="1:26" ht="15">
+    <row r="39" spans="1:26" ht="15" hidden="1">
       <c r="A39" t="s">
         <v>256</v>
       </c>
@@ -10090,7 +10075,7 @@
         <v>32</v>
       </c>
     </row>
-    <row r="40" spans="1:26" ht="15">
+    <row r="40" spans="1:26" ht="15" hidden="1">
       <c r="A40" t="s">
         <v>265</v>
       </c>
@@ -10170,7 +10155,7 @@
         <v>32</v>
       </c>
     </row>
-    <row r="41" spans="1:26" ht="15">
+    <row r="41" spans="1:26" ht="15" hidden="1">
       <c r="A41" s="1">
         <v>46177.584027777775</v>
       </c>
@@ -10250,7 +10235,7 @@
         <v>276</v>
       </c>
     </row>
-    <row r="42" spans="1:26" ht="15">
+    <row r="42" spans="1:26" ht="15" hidden="1">
       <c r="A42" t="s">
         <v>277</v>
       </c>
@@ -10330,7 +10315,7 @@
         <v>276</v>
       </c>
     </row>
-    <row r="43" spans="1:26" ht="15">
+    <row r="43" spans="1:26" ht="15" hidden="1">
       <c r="A43" s="1">
         <v>46147.499305555553</v>
       </c>
@@ -10410,7 +10395,7 @@
         <v>276</v>
       </c>
     </row>
-    <row r="44" spans="1:26" ht="15">
+    <row r="44" spans="1:26" ht="15" hidden="1">
       <c r="A44" t="s">
         <v>284</v>
       </c>
@@ -10490,7 +10475,7 @@
         <v>276</v>
       </c>
     </row>
-    <row r="45" spans="1:26" ht="15">
+    <row r="45" spans="1:26" ht="15" hidden="1">
       <c r="A45" s="1">
         <v>46177.533333333333</v>
       </c>
@@ -10570,7 +10555,7 @@
         <v>297</v>
       </c>
     </row>
-    <row r="46" spans="1:26" ht="15">
+    <row r="46" spans="1:26" ht="15" hidden="1">
       <c r="A46" t="s">
         <v>298</v>
       </c>
@@ -10650,7 +10635,7 @@
         <v>297</v>
       </c>
     </row>
-    <row r="47" spans="1:26" ht="15">
+    <row r="47" spans="1:26" ht="15" hidden="1">
       <c r="A47" t="s">
         <v>305</v>
       </c>
@@ -10730,7 +10715,7 @@
         <v>297</v>
       </c>
     </row>
-    <row r="48" spans="1:26" ht="15">
+    <row r="48" spans="1:26" ht="15" hidden="1">
       <c r="A48" s="1">
         <v>46056.451388888891</v>
       </c>
@@ -10810,7 +10795,7 @@
         <v>246</v>
       </c>
     </row>
-    <row r="49" spans="1:26" ht="15">
+    <row r="49" spans="1:26" ht="15" hidden="1">
       <c r="A49" t="s">
         <v>315</v>
       </c>
@@ -10890,7 +10875,7 @@
         <v>246</v>
       </c>
     </row>
-    <row r="50" spans="1:26" ht="15">
+    <row r="50" spans="1:26" ht="15" hidden="1">
       <c r="A50" t="s">
         <v>322</v>
       </c>
@@ -10970,7 +10955,7 @@
         <v>246</v>
       </c>
     </row>
-    <row r="51" spans="1:26" ht="15">
+    <row r="51" spans="1:26" ht="15" hidden="1">
       <c r="A51" t="s">
         <v>328</v>
       </c>
@@ -11050,7 +11035,7 @@
         <v>246</v>
       </c>
     </row>
-    <row r="52" spans="1:26" ht="15">
+    <row r="52" spans="1:26" ht="15" hidden="1">
       <c r="A52" t="s">
         <v>336</v>
       </c>
@@ -11130,7 +11115,7 @@
         <v>246</v>
       </c>
     </row>
-    <row r="53" spans="1:26" ht="15">
+    <row r="53" spans="1:26" ht="15" hidden="1">
       <c r="A53" t="s">
         <v>342</v>
       </c>
@@ -11210,7 +11195,7 @@
         <v>246</v>
       </c>
     </row>
-    <row r="54" spans="1:26" ht="15">
+    <row r="54" spans="1:26" ht="15" hidden="1">
       <c r="A54" t="s">
         <v>349</v>
       </c>
@@ -11290,7 +11275,7 @@
         <v>246</v>
       </c>
     </row>
-    <row r="55" spans="1:26" ht="15">
+    <row r="55" spans="1:26" ht="15" hidden="1">
       <c r="A55" t="s">
         <v>358</v>
       </c>
@@ -11370,7 +11355,7 @@
         <v>225</v>
       </c>
     </row>
-    <row r="56" spans="1:26" ht="15">
+    <row r="56" spans="1:26" ht="15" hidden="1">
       <c r="A56" t="s">
         <v>367</v>
       </c>
@@ -11450,7 +11435,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="57" spans="1:26" ht="15">
+    <row r="57" spans="1:26" ht="15" hidden="1">
       <c r="A57" t="s">
         <v>377</v>
       </c>
@@ -11530,7 +11515,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="58" spans="1:26" ht="15">
+    <row r="58" spans="1:26" ht="15" hidden="1">
       <c r="A58" t="s">
         <v>386</v>
       </c>
@@ -11610,7 +11595,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="59" spans="1:26" ht="29.25">
+    <row r="59" spans="1:26" ht="29.25" hidden="1">
       <c r="A59" s="1">
         <v>46028.415972222225</v>
       </c>
@@ -11690,7 +11675,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="60" spans="1:26" ht="15">
+    <row r="60" spans="1:26" ht="15" hidden="1">
       <c r="A60" t="s">
         <v>402</v>
       </c>
@@ -11770,7 +11755,7 @@
         <v>246</v>
       </c>
     </row>
-    <row r="61" spans="1:26" ht="15">
+    <row r="61" spans="1:26" ht="15" hidden="1">
       <c r="A61" t="s">
         <v>409</v>
       </c>
@@ -11850,7 +11835,7 @@
         <v>246</v>
       </c>
     </row>
-    <row r="62" spans="1:26" ht="15">
+    <row r="62" spans="1:26" ht="15" hidden="1">
       <c r="A62" s="1">
         <v>46300.675694444442</v>
       </c>
@@ -11930,7 +11915,7 @@
         <v>246</v>
       </c>
     </row>
-    <row r="63" spans="1:26" ht="15">
+    <row r="63" spans="1:26" ht="15" hidden="1">
       <c r="A63" t="s">
         <v>420</v>
       </c>
@@ -12010,7 +11995,7 @@
         <v>32</v>
       </c>
     </row>
-    <row r="64" spans="1:26" ht="15">
+    <row r="64" spans="1:26" ht="15" hidden="1">
       <c r="A64" t="s">
         <v>427</v>
       </c>
@@ -12090,7 +12075,7 @@
         <v>436</v>
       </c>
     </row>
-    <row r="65" spans="1:26" ht="15">
+    <row r="65" spans="1:26" ht="15" hidden="1">
       <c r="A65" s="1">
         <v>46297.706944444442</v>
       </c>
@@ -12170,7 +12155,7 @@
         <v>436</v>
       </c>
     </row>
-    <row r="66" spans="1:26" ht="15">
+    <row r="66" spans="1:26" ht="15" hidden="1">
       <c r="A66" s="1">
         <v>46239.543749999997</v>
       </c>
@@ -12250,7 +12235,7 @@
         <v>436</v>
       </c>
     </row>
-    <row r="67" spans="1:26" ht="15">
+    <row r="67" spans="1:26" ht="15" hidden="1">
       <c r="A67" t="s">
         <v>449</v>
       </c>
@@ -12330,7 +12315,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="68" spans="1:26" ht="15">
+    <row r="68" spans="1:26" ht="15" hidden="1">
       <c r="A68" t="s">
         <v>455</v>
       </c>
@@ -12410,7 +12395,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="69" spans="1:26" ht="15">
+    <row r="69" spans="1:26" ht="15" hidden="1">
       <c r="A69" s="1">
         <v>46116.837500000001</v>
       </c>
@@ -12490,7 +12475,7 @@
         <v>225</v>
       </c>
     </row>
-    <row r="70" spans="1:26" ht="15">
+    <row r="70" spans="1:26" ht="15" hidden="1">
       <c r="A70" s="1">
         <v>46026.467361111114</v>
       </c>
@@ -12570,7 +12555,7 @@
         <v>32</v>
       </c>
     </row>
-    <row r="71" spans="1:26" ht="15">
+    <row r="71" spans="1:26" ht="15" hidden="1">
       <c r="A71" s="1">
         <v>46238.624305555553</v>
       </c>
@@ -12650,7 +12635,7 @@
         <v>32</v>
       </c>
     </row>
-    <row r="72" spans="1:26" ht="15">
+    <row r="72" spans="1:26" ht="15" hidden="1">
       <c r="A72" t="s">
         <v>478</v>
       </c>
@@ -12730,7 +12715,7 @@
         <v>32</v>
       </c>
     </row>
-    <row r="73" spans="1:26" ht="15">
+    <row r="73" spans="1:26" ht="15" hidden="1">
       <c r="A73" s="1">
         <v>46239.632638888892</v>
       </c>
@@ -12810,7 +12795,7 @@
         <v>32</v>
       </c>
     </row>
-    <row r="74" spans="1:26" ht="15">
+    <row r="74" spans="1:26" ht="15" hidden="1">
       <c r="A74" s="1">
         <v>46239.643055555556</v>
       </c>
@@ -12890,7 +12875,7 @@
         <v>32</v>
       </c>
     </row>
-    <row r="75" spans="1:26" ht="15">
+    <row r="75" spans="1:26" ht="15" hidden="1">
       <c r="A75" t="s">
         <v>491</v>
       </c>
@@ -12970,7 +12955,7 @@
         <v>32</v>
       </c>
     </row>
-    <row r="76" spans="1:26" ht="15">
+    <row r="76" spans="1:26" ht="15" hidden="1">
       <c r="A76" t="s">
         <v>496</v>
       </c>
@@ -13050,7 +13035,7 @@
         <v>32</v>
       </c>
     </row>
-    <row r="77" spans="1:26" ht="15">
+    <row r="77" spans="1:26" ht="15" hidden="1">
       <c r="A77" t="s">
         <v>502</v>
       </c>
@@ -13130,7 +13115,7 @@
         <v>32</v>
       </c>
     </row>
-    <row r="78" spans="1:26" ht="15">
+    <row r="78" spans="1:26" ht="15" hidden="1">
       <c r="A78" t="s">
         <v>506</v>
       </c>
@@ -13530,7 +13515,7 @@
         <v>518</v>
       </c>
     </row>
-    <row r="83" spans="1:26" ht="15">
+    <row r="83" spans="1:26" ht="15" hidden="1">
       <c r="A83" s="1">
         <v>46269.668055555558</v>
       </c>
@@ -13610,7 +13595,7 @@
         <v>436</v>
       </c>
     </row>
-    <row r="84" spans="1:26" ht="15">
+    <row r="84" spans="1:26" ht="15" hidden="1">
       <c r="A84" s="1">
         <v>46117.512499999997</v>
       </c>
@@ -13690,7 +13675,7 @@
         <v>436</v>
       </c>
     </row>
-    <row r="85" spans="1:26" ht="15">
+    <row r="85" spans="1:26" ht="15" hidden="1">
       <c r="A85" s="1">
         <v>46299.574305555558</v>
       </c>
@@ -13770,7 +13755,7 @@
         <v>436</v>
       </c>
     </row>
-    <row r="86" spans="1:26" ht="15">
+    <row r="86" spans="1:26" ht="15" hidden="1">
       <c r="A86" t="s">
         <v>560</v>
       </c>
@@ -13850,7 +13835,7 @@
         <v>436</v>
       </c>
     </row>
-    <row r="87" spans="1:26" ht="15">
+    <row r="87" spans="1:26" ht="15" hidden="1">
       <c r="A87" t="s">
         <v>567</v>
       </c>
@@ -13930,7 +13915,7 @@
         <v>436</v>
       </c>
     </row>
-    <row r="88" spans="1:26" ht="15">
+    <row r="88" spans="1:26" ht="15" hidden="1">
       <c r="A88" s="1">
         <v>46117.518055555556</v>
       </c>
@@ -14010,7 +13995,7 @@
         <v>436</v>
       </c>
     </row>
-    <row r="89" spans="1:26" ht="15">
+    <row r="89" spans="1:26" ht="15" hidden="1">
       <c r="A89" t="s">
         <v>577</v>
       </c>
@@ -14090,7 +14075,7 @@
         <v>436</v>
       </c>
     </row>
-    <row r="90" spans="1:26" ht="15">
+    <row r="90" spans="1:26" ht="15" hidden="1">
       <c r="A90" t="s">
         <v>582</v>
       </c>
@@ -14170,7 +14155,7 @@
         <v>436</v>
       </c>
     </row>
-    <row r="91" spans="1:26" ht="15">
+    <row r="91" spans="1:26" ht="15" hidden="1">
       <c r="A91" t="s">
         <v>588</v>
       </c>
@@ -14250,7 +14235,7 @@
         <v>436</v>
       </c>
     </row>
-    <row r="92" spans="1:26" ht="15">
+    <row r="92" spans="1:26" ht="15" hidden="1">
       <c r="A92" t="s">
         <v>593</v>
       </c>
@@ -14330,7 +14315,7 @@
         <v>225</v>
       </c>
     </row>
-    <row r="93" spans="1:26" ht="15">
+    <row r="93" spans="1:26" ht="15" hidden="1">
       <c r="A93" s="1">
         <v>46028.518750000003</v>
       </c>
@@ -14810,7 +14795,7 @@
         <v>518</v>
       </c>
     </row>
-    <row r="99" spans="1:26" ht="15">
+    <row r="99" spans="1:26" ht="15" hidden="1">
       <c r="A99" t="s">
         <v>625</v>
       </c>
@@ -14890,7 +14875,7 @@
         <v>246</v>
       </c>
     </row>
-    <row r="100" spans="1:26" ht="15">
+    <row r="100" spans="1:26" ht="15" hidden="1">
       <c r="A100" t="s">
         <v>634</v>
       </c>
@@ -14970,7 +14955,7 @@
         <v>246</v>
       </c>
     </row>
-    <row r="101" spans="1:26" ht="15">
+    <row r="101" spans="1:26" ht="15" hidden="1">
       <c r="A101" s="1">
         <v>46116.497916666667</v>
       </c>
@@ -15050,7 +15035,7 @@
         <v>246</v>
       </c>
     </row>
-    <row r="102" spans="1:26" ht="15">
+    <row r="102" spans="1:26" ht="15" hidden="1">
       <c r="A102" t="s">
         <v>644</v>
       </c>
@@ -15130,7 +15115,7 @@
         <v>246</v>
       </c>
     </row>
-    <row r="103" spans="1:26" ht="15">
+    <row r="103" spans="1:26" ht="15" hidden="1">
       <c r="A103" t="s">
         <v>649</v>
       </c>
@@ -15210,7 +15195,7 @@
         <v>297</v>
       </c>
     </row>
-    <row r="104" spans="1:26" ht="15">
+    <row r="104" spans="1:26" ht="15" hidden="1">
       <c r="A104" t="s">
         <v>657</v>
       </c>
@@ -15290,7 +15275,7 @@
         <v>297</v>
       </c>
     </row>
-    <row r="105" spans="1:26" ht="15">
+    <row r="105" spans="1:26" ht="15" hidden="1">
       <c r="A105" t="s">
         <v>662</v>
       </c>
@@ -15370,7 +15355,7 @@
         <v>297</v>
       </c>
     </row>
-    <row r="106" spans="1:26" ht="15">
+    <row r="106" spans="1:26" ht="15" hidden="1">
       <c r="A106" t="s">
         <v>665</v>
       </c>
@@ -15450,7 +15435,7 @@
         <v>297</v>
       </c>
     </row>
-    <row r="107" spans="1:26" ht="15">
+    <row r="107" spans="1:26" ht="15" hidden="1">
       <c r="A107" t="s">
         <v>668</v>
       </c>
@@ -15530,7 +15515,7 @@
         <v>297</v>
       </c>
     </row>
-    <row r="108" spans="1:26" ht="15">
+    <row r="108" spans="1:26" ht="15" hidden="1">
       <c r="A108" t="s">
         <v>671</v>
       </c>
@@ -15610,7 +15595,7 @@
         <v>297</v>
       </c>
     </row>
-    <row r="109" spans="1:26" ht="15">
+    <row r="109" spans="1:26" ht="15" hidden="1">
       <c r="A109" t="s">
         <v>674</v>
       </c>
@@ -15690,7 +15675,7 @@
         <v>297</v>
       </c>
     </row>
-    <row r="110" spans="1:26" ht="15">
+    <row r="110" spans="1:26" ht="15" hidden="1">
       <c r="A110" t="s">
         <v>677</v>
       </c>
@@ -15770,7 +15755,7 @@
         <v>297</v>
       </c>
     </row>
-    <row r="111" spans="1:26" ht="15">
+    <row r="111" spans="1:26" ht="15" hidden="1">
       <c r="A111" t="s">
         <v>680</v>
       </c>
@@ -15850,7 +15835,7 @@
         <v>297</v>
       </c>
     </row>
-    <row r="112" spans="1:26" ht="15">
+    <row r="112" spans="1:26" ht="15" hidden="1">
       <c r="A112" s="1">
         <v>46271.526388888888</v>
       </c>
@@ -15930,7 +15915,7 @@
         <v>297</v>
       </c>
     </row>
-    <row r="113" spans="1:26" ht="15">
+    <row r="113" spans="1:26" ht="15" hidden="1">
       <c r="A113" s="1">
         <v>46271.53402777778</v>
       </c>
@@ -16010,7 +15995,7 @@
         <v>297</v>
       </c>
     </row>
-    <row r="114" spans="1:26" ht="15">
+    <row r="114" spans="1:26" ht="15" hidden="1">
       <c r="A114" s="1">
         <v>46271.538194444445</v>
       </c>
@@ -16090,7 +16075,7 @@
         <v>297</v>
       </c>
     </row>
-    <row r="115" spans="1:26" ht="15">
+    <row r="115" spans="1:26" ht="15" hidden="1">
       <c r="A115" t="s">
         <v>689</v>
       </c>
@@ -16170,7 +16155,7 @@
         <v>297</v>
       </c>
     </row>
-    <row r="116" spans="1:26" ht="15">
+    <row r="116" spans="1:26" ht="15" hidden="1">
       <c r="A116" t="s">
         <v>693</v>
       </c>
@@ -16250,7 +16235,7 @@
         <v>297</v>
       </c>
     </row>
-    <row r="117" spans="1:26" ht="15">
+    <row r="117" spans="1:26" ht="15" hidden="1">
       <c r="A117" t="s">
         <v>696</v>
       </c>
@@ -16330,7 +16315,7 @@
         <v>297</v>
       </c>
     </row>
-    <row r="118" spans="1:26" ht="15">
+    <row r="118" spans="1:26" ht="15" hidden="1">
       <c r="A118" t="s">
         <v>699</v>
       </c>
@@ -16410,7 +16395,7 @@
         <v>297</v>
       </c>
     </row>
-    <row r="119" spans="1:26" ht="15">
+    <row r="119" spans="1:26" ht="15" hidden="1">
       <c r="A119" t="s">
         <v>702</v>
       </c>
@@ -16490,7 +16475,7 @@
         <v>297</v>
       </c>
     </row>
-    <row r="120" spans="1:26" ht="15">
+    <row r="120" spans="1:26" ht="15" hidden="1">
       <c r="A120" t="s">
         <v>705</v>
       </c>
@@ -16570,7 +16555,7 @@
         <v>297</v>
       </c>
     </row>
-    <row r="121" spans="1:26" ht="15">
+    <row r="121" spans="1:26" ht="15" hidden="1">
       <c r="A121" t="s">
         <v>708</v>
       </c>
@@ -16650,7 +16635,7 @@
         <v>297</v>
       </c>
     </row>
-    <row r="122" spans="1:26" ht="15">
+    <row r="122" spans="1:26" ht="15" hidden="1">
       <c r="A122" t="s">
         <v>711</v>
       </c>
@@ -16730,7 +16715,7 @@
         <v>297</v>
       </c>
     </row>
-    <row r="123" spans="1:26" ht="15">
+    <row r="123" spans="1:26" ht="15" hidden="1">
       <c r="A123" s="1">
         <v>45932.425694444442</v>
       </c>
@@ -16810,7 +16795,7 @@
         <v>246</v>
       </c>
     </row>
-    <row r="124" spans="1:26" ht="15">
+    <row r="124" spans="1:26" ht="15" hidden="1">
       <c r="A124" t="s">
         <v>720</v>
       </c>
@@ -16890,7 +16875,7 @@
         <v>246</v>
       </c>
     </row>
-    <row r="125" spans="1:26" ht="15">
+    <row r="125" spans="1:26" ht="15" hidden="1">
       <c r="A125" t="s">
         <v>726</v>
       </c>
@@ -16970,7 +16955,7 @@
         <v>32</v>
       </c>
     </row>
-    <row r="126" spans="1:26" ht="15">
+    <row r="126" spans="1:26" ht="15" hidden="1">
       <c r="A126" t="s">
         <v>732</v>
       </c>
@@ -17050,7 +17035,7 @@
         <v>436</v>
       </c>
     </row>
-    <row r="127" spans="1:26" ht="15">
+    <row r="127" spans="1:26" ht="15" hidden="1">
       <c r="A127" t="s">
         <v>737</v>
       </c>
@@ -17130,7 +17115,7 @@
         <v>297</v>
       </c>
     </row>
-    <row r="128" spans="1:26" ht="15">
+    <row r="128" spans="1:26" ht="15" hidden="1">
       <c r="A128" t="s">
         <v>743</v>
       </c>
@@ -17210,7 +17195,7 @@
         <v>297</v>
       </c>
     </row>
-    <row r="129" spans="1:26" ht="15">
+    <row r="129" spans="1:26" ht="15" hidden="1">
       <c r="A129" t="s">
         <v>749</v>
       </c>
@@ -17290,7 +17275,7 @@
         <v>297</v>
       </c>
     </row>
-    <row r="130" spans="1:26" ht="15">
+    <row r="130" spans="1:26" ht="15" hidden="1">
       <c r="A130" t="s">
         <v>753</v>
       </c>
@@ -17370,7 +17355,7 @@
         <v>297</v>
       </c>
     </row>
-    <row r="131" spans="1:26" ht="15">
+    <row r="131" spans="1:26" ht="15" hidden="1">
       <c r="A131" t="s">
         <v>759</v>
       </c>
@@ -17450,7 +17435,7 @@
         <v>246</v>
       </c>
     </row>
-    <row r="132" spans="1:26" ht="15">
+    <row r="132" spans="1:26" ht="15" hidden="1">
       <c r="A132" t="s">
         <v>767</v>
       </c>
@@ -17530,7 +17515,7 @@
         <v>246</v>
       </c>
     </row>
-    <row r="133" spans="1:26" ht="15">
+    <row r="133" spans="1:26" ht="15" hidden="1">
       <c r="A133" t="s">
         <v>774</v>
       </c>
@@ -17610,7 +17595,7 @@
         <v>246</v>
       </c>
     </row>
-    <row r="134" spans="1:26" ht="15">
+    <row r="134" spans="1:26" ht="15" hidden="1">
       <c r="A134" t="s">
         <v>781</v>
       </c>
@@ -17690,7 +17675,7 @@
         <v>246</v>
       </c>
     </row>
-    <row r="135" spans="1:26" ht="15">
+    <row r="135" spans="1:26" ht="15" hidden="1">
       <c r="A135" s="1">
         <v>46207.655555555553</v>
       </c>
@@ -17770,7 +17755,7 @@
         <v>246</v>
       </c>
     </row>
-    <row r="136" spans="1:26" ht="15">
+    <row r="136" spans="1:26" ht="15" hidden="1">
       <c r="A136" s="1">
         <v>46207.675000000003</v>
       </c>
@@ -17850,7 +17835,7 @@
         <v>246</v>
       </c>
     </row>
-    <row r="137" spans="1:26" ht="15">
+    <row r="137" spans="1:26" ht="15" hidden="1">
       <c r="A137" s="1">
         <v>46238.697916666664</v>
       </c>
@@ -17930,7 +17915,7 @@
         <v>246</v>
       </c>
     </row>
-    <row r="138" spans="1:26" ht="15">
+    <row r="138" spans="1:26" ht="15" hidden="1">
       <c r="A138" s="1">
         <v>46238.70416666667</v>
       </c>
@@ -18010,7 +17995,7 @@
         <v>246</v>
       </c>
     </row>
-    <row r="139" spans="1:26" ht="15">
+    <row r="139" spans="1:26" ht="15" hidden="1">
       <c r="A139" s="1">
         <v>46238.706944444442</v>
       </c>
@@ -18090,7 +18075,7 @@
         <v>246</v>
       </c>
     </row>
-    <row r="140" spans="1:26" ht="15">
+    <row r="140" spans="1:26" ht="15" hidden="1">
       <c r="A140" s="1">
         <v>46238.711111111108</v>
       </c>
@@ -18170,7 +18155,7 @@
         <v>246</v>
       </c>
     </row>
-    <row r="141" spans="1:26" ht="15">
+    <row r="141" spans="1:26" ht="15" hidden="1">
       <c r="A141" s="1">
         <v>46238.731944444444</v>
       </c>
@@ -18250,7 +18235,7 @@
         <v>246</v>
       </c>
     </row>
-    <row r="142" spans="1:26" ht="15">
+    <row r="142" spans="1:26" ht="15" hidden="1">
       <c r="A142" s="1">
         <v>46269.700694444444</v>
       </c>
@@ -18330,7 +18315,7 @@
         <v>246</v>
       </c>
     </row>
-    <row r="143" spans="1:26" ht="15">
+    <row r="143" spans="1:26" ht="15" hidden="1">
       <c r="A143" s="1">
         <v>46269.711111111108</v>
       </c>
@@ -18410,7 +18395,7 @@
         <v>246</v>
       </c>
     </row>
-    <row r="144" spans="1:26" ht="15">
+    <row r="144" spans="1:26" ht="15" hidden="1">
       <c r="A144" s="1">
         <v>46269.717361111114</v>
       </c>
@@ -18490,7 +18475,7 @@
         <v>246</v>
       </c>
     </row>
-    <row r="145" spans="1:26" ht="15">
+    <row r="145" spans="1:26" ht="15" hidden="1">
       <c r="A145" s="1">
         <v>46269.738888888889</v>
       </c>
@@ -18570,7 +18555,7 @@
         <v>246</v>
       </c>
     </row>
-    <row r="146" spans="1:26" ht="15">
+    <row r="146" spans="1:26" ht="15" hidden="1">
       <c r="A146" s="1">
         <v>46299.675694444442</v>
       </c>
@@ -18650,7 +18635,7 @@
         <v>246</v>
       </c>
     </row>
-    <row r="147" spans="1:26" ht="15">
+    <row r="147" spans="1:26" ht="15" hidden="1">
       <c r="A147" s="1">
         <v>46299.695138888892</v>
       </c>
@@ -18730,7 +18715,7 @@
         <v>246</v>
       </c>
     </row>
-    <row r="148" spans="1:26" ht="15">
+    <row r="148" spans="1:26" ht="15" hidden="1">
       <c r="A148" s="1">
         <v>46299.709722222222</v>
       </c>
@@ -18810,7 +18795,7 @@
         <v>246</v>
       </c>
     </row>
-    <row r="149" spans="1:26" ht="15">
+    <row r="149" spans="1:26" ht="15" hidden="1">
       <c r="A149" s="1">
         <v>46299.713194444441</v>
       </c>
@@ -18890,7 +18875,7 @@
         <v>246</v>
       </c>
     </row>
-    <row r="150" spans="1:26" ht="15">
+    <row r="150" spans="1:26" ht="15" hidden="1">
       <c r="A150" s="1">
         <v>46299.718055555553</v>
       </c>
@@ -18970,7 +18955,7 @@
         <v>246</v>
       </c>
     </row>
-    <row r="151" spans="1:26" ht="15">
+    <row r="151" spans="1:26" ht="15" hidden="1">
       <c r="A151" s="1">
         <v>46299.722222222219</v>
       </c>
@@ -19050,7 +19035,7 @@
         <v>246</v>
       </c>
     </row>
-    <row r="152" spans="1:26" ht="15">
+    <row r="152" spans="1:26" ht="15" hidden="1">
       <c r="A152" s="1">
         <v>46299.725694444445</v>
       </c>
@@ -19130,7 +19115,7 @@
         <v>246</v>
       </c>
     </row>
-    <row r="153" spans="1:26" ht="15">
+    <row r="153" spans="1:26" ht="15" hidden="1">
       <c r="A153" t="s">
         <v>843</v>
       </c>
@@ -19210,7 +19195,7 @@
         <v>246</v>
       </c>
     </row>
-    <row r="154" spans="1:26" ht="15">
+    <row r="154" spans="1:26" ht="15" hidden="1">
       <c r="A154" t="s">
         <v>847</v>
       </c>
@@ -19290,7 +19275,7 @@
         <v>246</v>
       </c>
     </row>
-    <row r="155" spans="1:26" ht="15">
+    <row r="155" spans="1:26" ht="15" hidden="1">
       <c r="A155" t="s">
         <v>851</v>
       </c>
@@ -19370,7 +19355,7 @@
         <v>246</v>
       </c>
     </row>
-    <row r="156" spans="1:26" ht="15">
+    <row r="156" spans="1:26" ht="15" hidden="1">
       <c r="A156" t="s">
         <v>856</v>
       </c>
@@ -19450,7 +19435,7 @@
         <v>246</v>
       </c>
     </row>
-    <row r="157" spans="1:26" ht="15">
+    <row r="157" spans="1:26" ht="15" hidden="1">
       <c r="A157" t="s">
         <v>860</v>
       </c>
@@ -19530,7 +19515,7 @@
         <v>246</v>
       </c>
     </row>
-    <row r="158" spans="1:26" ht="15">
+    <row r="158" spans="1:26" ht="15" hidden="1">
       <c r="A158" t="s">
         <v>865</v>
       </c>
@@ -19610,7 +19595,7 @@
         <v>246</v>
       </c>
     </row>
-    <row r="159" spans="1:26" ht="15">
+    <row r="159" spans="1:26" ht="15" hidden="1">
       <c r="A159" t="s">
         <v>869</v>
       </c>
@@ -19690,7 +19675,7 @@
         <v>246</v>
       </c>
     </row>
-    <row r="160" spans="1:26" ht="15">
+    <row r="160" spans="1:26" ht="15" hidden="1">
       <c r="A160" t="s">
         <v>873</v>
       </c>
@@ -19770,7 +19755,7 @@
         <v>246</v>
       </c>
     </row>
-    <row r="161" spans="1:26" ht="15">
+    <row r="161" spans="1:26" ht="15" hidden="1">
       <c r="A161" t="s">
         <v>878</v>
       </c>
@@ -19850,7 +19835,7 @@
         <v>246</v>
       </c>
     </row>
-    <row r="162" spans="1:26" ht="15">
+    <row r="162" spans="1:26" ht="15" hidden="1">
       <c r="A162" s="1">
         <v>46147.706944444442</v>
       </c>
@@ -19930,7 +19915,7 @@
         <v>246</v>
       </c>
     </row>
-    <row r="163" spans="1:26" ht="15">
+    <row r="163" spans="1:26" ht="15" hidden="1">
       <c r="A163" s="1">
         <v>46270.556250000001</v>
       </c>
@@ -20010,7 +19995,7 @@
         <v>246</v>
       </c>
     </row>
-    <row r="164" spans="1:26" ht="15">
+    <row r="164" spans="1:26" ht="15" hidden="1">
       <c r="A164" s="1">
         <v>46270.55972222222</v>
       </c>
@@ -20090,7 +20075,7 @@
         <v>246</v>
       </c>
     </row>
-    <row r="165" spans="1:26" ht="15">
+    <row r="165" spans="1:26" ht="15" hidden="1">
       <c r="A165" t="s">
         <v>895</v>
       </c>
@@ -20170,7 +20155,7 @@
         <v>246</v>
       </c>
     </row>
-    <row r="166" spans="1:26" ht="15">
+    <row r="166" spans="1:26" ht="15" hidden="1">
       <c r="A166" t="s">
         <v>899</v>
       </c>
@@ -20250,7 +20235,7 @@
         <v>246</v>
       </c>
     </row>
-    <row r="167" spans="1:26" ht="15">
+    <row r="167" spans="1:26" ht="15" hidden="1">
       <c r="A167" t="s">
         <v>903</v>
       </c>
@@ -20330,7 +20315,7 @@
         <v>246</v>
       </c>
     </row>
-    <row r="168" spans="1:26" ht="15">
+    <row r="168" spans="1:26" ht="15" hidden="1">
       <c r="A168" t="s">
         <v>907</v>
       </c>
@@ -20410,7 +20395,7 @@
         <v>246</v>
       </c>
     </row>
-    <row r="169" spans="1:26" ht="15">
+    <row r="169" spans="1:26" ht="15" hidden="1">
       <c r="A169" s="1">
         <v>46267.501388888886</v>
       </c>
@@ -20490,7 +20475,7 @@
         <v>246</v>
       </c>
     </row>
-    <row r="170" spans="1:26" ht="15">
+    <row r="170" spans="1:26" ht="15" hidden="1">
       <c r="A170" t="s">
         <v>915</v>
       </c>
@@ -20570,7 +20555,7 @@
         <v>246</v>
       </c>
     </row>
-    <row r="171" spans="1:26" ht="15">
+    <row r="171" spans="1:26" ht="15" hidden="1">
       <c r="A171" t="s">
         <v>919</v>
       </c>
@@ -20650,7 +20635,7 @@
         <v>246</v>
       </c>
     </row>
-    <row r="172" spans="1:26" ht="15">
+    <row r="172" spans="1:26" ht="15" hidden="1">
       <c r="A172" t="s">
         <v>923</v>
       </c>
@@ -20730,7 +20715,7 @@
         <v>246</v>
       </c>
     </row>
-    <row r="173" spans="1:26" ht="15">
+    <row r="173" spans="1:26" ht="15" hidden="1">
       <c r="A173" t="s">
         <v>927</v>
       </c>
@@ -20810,7 +20795,7 @@
         <v>246</v>
       </c>
     </row>
-    <row r="174" spans="1:26" ht="15">
+    <row r="174" spans="1:26" ht="15" hidden="1">
       <c r="A174" t="s">
         <v>931</v>
       </c>
@@ -20890,7 +20875,7 @@
         <v>246</v>
       </c>
     </row>
-    <row r="175" spans="1:26" ht="15">
+    <row r="175" spans="1:26" ht="15" hidden="1">
       <c r="A175" t="s">
         <v>935</v>
       </c>
@@ -20970,7 +20955,7 @@
         <v>246</v>
       </c>
     </row>
-    <row r="176" spans="1:26" ht="15">
+    <row r="176" spans="1:26" ht="15" hidden="1">
       <c r="A176" t="s">
         <v>939</v>
       </c>
@@ -21050,7 +21035,7 @@
         <v>246</v>
       </c>
     </row>
-    <row r="177" spans="1:26" ht="15">
+    <row r="177" spans="1:26" ht="15" hidden="1">
       <c r="A177" t="s">
         <v>943</v>
       </c>
@@ -21130,7 +21115,7 @@
         <v>246</v>
       </c>
     </row>
-    <row r="178" spans="1:26" ht="15">
+    <row r="178" spans="1:26" ht="15" hidden="1">
       <c r="A178" t="s">
         <v>947</v>
       </c>
@@ -21210,7 +21195,7 @@
         <v>246</v>
       </c>
     </row>
-    <row r="179" spans="1:26" ht="15">
+    <row r="179" spans="1:26" ht="15" hidden="1">
       <c r="A179" t="s">
         <v>952</v>
       </c>
@@ -21290,7 +21275,7 @@
         <v>246</v>
       </c>
     </row>
-    <row r="180" spans="1:26" ht="15">
+    <row r="180" spans="1:26" ht="15" hidden="1">
       <c r="A180" t="s">
         <v>956</v>
       </c>
@@ -21370,7 +21355,7 @@
         <v>246</v>
       </c>
     </row>
-    <row r="181" spans="1:26" ht="15">
+    <row r="181" spans="1:26" ht="15" hidden="1">
       <c r="A181" t="s">
         <v>960</v>
       </c>
@@ -21450,7 +21435,7 @@
         <v>246</v>
       </c>
     </row>
-    <row r="182" spans="1:26" ht="15">
+    <row r="182" spans="1:26" ht="15" hidden="1">
       <c r="A182" t="s">
         <v>964</v>
       </c>
@@ -21530,7 +21515,7 @@
         <v>246</v>
       </c>
     </row>
-    <row r="183" spans="1:26" ht="15">
+    <row r="183" spans="1:26" ht="15" hidden="1">
       <c r="A183" t="s">
         <v>968</v>
       </c>
@@ -21610,7 +21595,7 @@
         <v>246</v>
       </c>
     </row>
-    <row r="184" spans="1:26" ht="15">
+    <row r="184" spans="1:26" ht="15" hidden="1">
       <c r="A184" t="s">
         <v>972</v>
       </c>
@@ -21690,7 +21675,7 @@
         <v>246</v>
       </c>
     </row>
-    <row r="185" spans="1:26" ht="15">
+    <row r="185" spans="1:26" ht="15" hidden="1">
       <c r="A185" t="s">
         <v>976</v>
       </c>
@@ -21770,7 +21755,7 @@
         <v>246</v>
       </c>
     </row>
-    <row r="186" spans="1:26" ht="15">
+    <row r="186" spans="1:26" ht="15" hidden="1">
       <c r="A186" t="s">
         <v>979</v>
       </c>
@@ -21850,7 +21835,7 @@
         <v>246</v>
       </c>
     </row>
-    <row r="187" spans="1:26" ht="15">
+    <row r="187" spans="1:26" ht="15" hidden="1">
       <c r="A187" s="1">
         <v>46028.713888888888</v>
       </c>
@@ -21930,7 +21915,7 @@
         <v>246</v>
       </c>
     </row>
-    <row r="188" spans="1:26" ht="15">
+    <row r="188" spans="1:26" ht="15" hidden="1">
       <c r="A188" t="s">
         <v>986</v>
       </c>
@@ -22010,7 +21995,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="189" spans="1:26" ht="15">
+    <row r="189" spans="1:26" ht="15" hidden="1">
       <c r="A189" s="1">
         <v>46332.530555555553</v>
       </c>
@@ -22090,7 +22075,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="190" spans="1:26" ht="15">
+    <row r="190" spans="1:26" ht="15" hidden="1">
       <c r="A190" t="s">
         <v>1003</v>
       </c>
@@ -22170,7 +22155,7 @@
         <v>436</v>
       </c>
     </row>
-    <row r="191" spans="1:26" ht="15">
+    <row r="191" spans="1:26" ht="15" hidden="1">
       <c r="A191" s="1">
         <v>45668.527777777781</v>
       </c>
@@ -22250,7 +22235,7 @@
         <v>225</v>
       </c>
     </row>
-    <row r="192" spans="1:26" ht="15">
+    <row r="192" spans="1:26" ht="15" hidden="1">
       <c r="A192" t="s">
         <v>1021</v>
       </c>
@@ -22330,7 +22315,7 @@
         <v>32</v>
       </c>
     </row>
-    <row r="193" spans="1:26" ht="15">
+    <row r="193" spans="1:26" ht="15" hidden="1">
       <c r="A193" s="1">
         <v>46332.667361111111</v>
       </c>
@@ -22410,7 +22395,7 @@
         <v>32</v>
       </c>
     </row>
-    <row r="194" spans="1:26" ht="15">
+    <row r="194" spans="1:26" ht="15" hidden="1">
       <c r="A194" s="1">
         <v>46329.643750000003</v>
       </c>
@@ -22490,7 +22475,7 @@
         <v>246</v>
       </c>
     </row>
-    <row r="195" spans="1:26" ht="15">
+    <row r="195" spans="1:26" ht="15" hidden="1">
       <c r="A195" t="s">
         <v>1037</v>
       </c>
@@ -22570,7 +22555,7 @@
         <v>246</v>
       </c>
     </row>
-    <row r="196" spans="1:26" ht="15">
+    <row r="196" spans="1:26" ht="15" hidden="1">
       <c r="A196" t="s">
         <v>1045</v>
       </c>
@@ -22650,7 +22635,7 @@
         <v>246</v>
       </c>
     </row>
-    <row r="197" spans="1:26" ht="15">
+    <row r="197" spans="1:26" ht="15" hidden="1">
       <c r="A197" s="1">
         <v>46059.475694444445</v>
       </c>
@@ -22730,7 +22715,7 @@
         <v>32</v>
       </c>
     </row>
-    <row r="198" spans="1:26" ht="15">
+    <row r="198" spans="1:26" ht="15" hidden="1">
       <c r="A198" s="1">
         <v>46301.53402777778</v>
       </c>
@@ -22810,7 +22795,7 @@
         <v>32</v>
       </c>
     </row>
-    <row r="199" spans="1:26" ht="15">
+    <row r="199" spans="1:26" ht="15" hidden="1">
       <c r="A199" t="s">
         <v>1066</v>
       </c>
@@ -22890,7 +22875,7 @@
         <v>32</v>
       </c>
     </row>
-    <row r="200" spans="1:26" ht="15">
+    <row r="200" spans="1:26" ht="15" hidden="1">
       <c r="A200" s="1">
         <v>46269.70416666667</v>
       </c>
@@ -22970,7 +22955,7 @@
         <v>32</v>
       </c>
     </row>
-    <row r="201" spans="1:26" ht="15">
+    <row r="201" spans="1:26" ht="15" hidden="1">
       <c r="A201" s="1">
         <v>46056.47152777778</v>
       </c>
@@ -23050,7 +23035,7 @@
         <v>246</v>
       </c>
     </row>
-    <row r="202" spans="1:26" ht="15">
+    <row r="202" spans="1:26" ht="15" hidden="1">
       <c r="A202" t="s">
         <v>1088</v>
       </c>
@@ -23130,7 +23115,7 @@
         <v>246</v>
       </c>
     </row>
-    <row r="203" spans="1:26" ht="15">
+    <row r="203" spans="1:26" ht="15" hidden="1">
       <c r="A203" t="s">
         <v>1094</v>
       </c>
@@ -23210,7 +23195,7 @@
         <v>246</v>
       </c>
     </row>
-    <row r="204" spans="1:26" ht="15">
+    <row r="204" spans="1:26" ht="15" hidden="1">
       <c r="A204" s="1">
         <v>46239.657638888886</v>
       </c>
@@ -23290,7 +23275,7 @@
         <v>246</v>
       </c>
     </row>
-    <row r="205" spans="1:26" ht="15">
+    <row r="205" spans="1:26" ht="15" hidden="1">
       <c r="A205" s="1">
         <v>46331.459027777775</v>
       </c>
@@ -23370,7 +23355,7 @@
         <v>246</v>
       </c>
     </row>
-    <row r="206" spans="1:26" ht="15">
+    <row r="206" spans="1:26" ht="15" hidden="1">
       <c r="A206" t="s">
         <v>1105</v>
       </c>
@@ -23450,7 +23435,7 @@
         <v>246</v>
       </c>
     </row>
-    <row r="207" spans="1:26" ht="15">
+    <row r="207" spans="1:26" ht="15" hidden="1">
       <c r="A207" s="1">
         <v>46332.488888888889</v>
       </c>
@@ -23530,7 +23515,7 @@
         <v>246</v>
       </c>
     </row>
-    <row r="208" spans="1:26" ht="15">
+    <row r="208" spans="1:26" ht="15" hidden="1">
       <c r="A208" t="s">
         <v>1111</v>
       </c>
@@ -23610,7 +23595,7 @@
         <v>246</v>
       </c>
     </row>
-    <row r="209" spans="1:26" ht="15">
+    <row r="209" spans="1:26" ht="15" hidden="1">
       <c r="A209" t="s">
         <v>1116</v>
       </c>
@@ -23690,7 +23675,7 @@
         <v>246</v>
       </c>
     </row>
-    <row r="210" spans="1:26" ht="15">
+    <row r="210" spans="1:26" ht="15" hidden="1">
       <c r="A210" s="1">
         <v>46144.847916666666</v>
       </c>
@@ -23770,7 +23755,7 @@
         <v>225</v>
       </c>
     </row>
-    <row r="211" spans="1:26" ht="15">
+    <row r="211" spans="1:26" ht="15" hidden="1">
       <c r="A211" s="1">
         <v>46056.472916666666</v>
       </c>
@@ -23850,7 +23835,7 @@
         <v>225</v>
       </c>
     </row>
-    <row r="212" spans="1:26" ht="15">
+    <row r="212" spans="1:26" ht="15" hidden="1">
       <c r="A212" s="1">
         <v>46237.95416666667</v>
       </c>
@@ -23930,7 +23915,7 @@
         <v>225</v>
       </c>
     </row>
-    <row r="213" spans="1:26" ht="15">
+    <row r="213" spans="1:26" ht="15" hidden="1">
       <c r="A213" t="s">
         <v>1132</v>
       </c>
@@ -24010,7 +23995,7 @@
         <v>225</v>
       </c>
     </row>
-    <row r="214" spans="1:26" ht="15">
+    <row r="214" spans="1:26" ht="15" hidden="1">
       <c r="A214" s="1">
         <v>46148.56527777778</v>
       </c>
@@ -24090,7 +24075,7 @@
         <v>225</v>
       </c>
     </row>
-    <row r="215" spans="1:26" ht="15">
+    <row r="215" spans="1:26" ht="15" hidden="1">
       <c r="A215" s="1">
         <v>46148.56527777778</v>
       </c>
@@ -24170,7 +24155,7 @@
         <v>225</v>
       </c>
     </row>
-    <row r="216" spans="1:26" ht="15">
+    <row r="216" spans="1:26" ht="15" hidden="1">
       <c r="A216" t="s">
         <v>1143</v>
       </c>
@@ -24730,7 +24715,7 @@
         <v>518</v>
       </c>
     </row>
-    <row r="223" spans="1:26" ht="15">
+    <row r="223" spans="1:26" ht="15" hidden="1">
       <c r="A223" t="s">
         <v>1186</v>
       </c>
@@ -24810,7 +24795,7 @@
         <v>436</v>
       </c>
     </row>
-    <row r="224" spans="1:26" ht="15">
+    <row r="224" spans="1:26" ht="15" hidden="1">
       <c r="A224" t="s">
         <v>1195</v>
       </c>
@@ -24970,7 +24955,7 @@
         <v>518</v>
       </c>
     </row>
-    <row r="226" spans="1:26" ht="15">
+    <row r="226" spans="1:26" ht="15" hidden="1">
       <c r="A226" t="s">
         <v>1206</v>
       </c>
@@ -25050,7 +25035,7 @@
         <v>1213</v>
       </c>
     </row>
-    <row r="227" spans="1:26" ht="15">
+    <row r="227" spans="1:26" ht="15" hidden="1">
       <c r="A227" s="1">
         <v>46296.427083333336</v>
       </c>
@@ -25130,7 +25115,7 @@
         <v>297</v>
       </c>
     </row>
-    <row r="228" spans="1:26" ht="15">
+    <row r="228" spans="1:26" ht="15" hidden="1">
       <c r="A228" s="1">
         <v>46205.686111111114</v>
       </c>
@@ -25210,7 +25195,7 @@
         <v>297</v>
       </c>
     </row>
-    <row r="229" spans="1:26" ht="15">
+    <row r="229" spans="1:26" ht="15" hidden="1">
       <c r="A229" s="1">
         <v>46268.555555555555</v>
       </c>
@@ -25290,7 +25275,7 @@
         <v>297</v>
       </c>
     </row>
-    <row r="230" spans="1:26" ht="15">
+    <row r="230" spans="1:26" ht="15" hidden="1">
       <c r="A230" t="s">
         <v>1232</v>
       </c>
@@ -25370,7 +25355,7 @@
         <v>1240</v>
       </c>
     </row>
-    <row r="231" spans="1:26" ht="15">
+    <row r="231" spans="1:26" ht="15" hidden="1">
       <c r="A231" t="s">
         <v>1241</v>
       </c>
@@ -25450,7 +25435,7 @@
         <v>436</v>
       </c>
     </row>
-    <row r="232" spans="1:26" ht="15">
+    <row r="232" spans="1:26" ht="15" hidden="1">
       <c r="A232" s="1">
         <v>46207.590277777781</v>
       </c>
@@ -25530,7 +25515,7 @@
         <v>436</v>
       </c>
     </row>
-    <row r="233" spans="1:26" ht="15">
+    <row r="233" spans="1:26" ht="15" hidden="1">
       <c r="A233" t="s">
         <v>1254</v>
       </c>
@@ -25610,7 +25595,7 @@
         <v>246</v>
       </c>
     </row>
-    <row r="234" spans="1:26" ht="15">
+    <row r="234" spans="1:26" ht="15" hidden="1">
       <c r="A234" s="1">
         <v>46028.749305555553</v>
       </c>
@@ -25690,7 +25675,7 @@
         <v>246</v>
       </c>
     </row>
-    <row r="235" spans="1:26" ht="15">
+    <row r="235" spans="1:26" ht="15" hidden="1">
       <c r="A235" t="s">
         <v>1266</v>
       </c>
@@ -25770,7 +25755,7 @@
         <v>246</v>
       </c>
     </row>
-    <row r="236" spans="1:26" ht="15">
+    <row r="236" spans="1:26" ht="15" hidden="1">
       <c r="A236" s="1">
         <v>46269.655555555553</v>
       </c>
@@ -25850,7 +25835,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="237" spans="1:26" ht="15">
+    <row r="237" spans="1:26" ht="15" hidden="1">
       <c r="A237" t="s">
         <v>1279</v>
       </c>
@@ -25930,7 +25915,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="238" spans="1:26" ht="15">
+    <row r="238" spans="1:26" ht="15" hidden="1">
       <c r="A238" t="s">
         <v>1284</v>
       </c>
@@ -26010,7 +25995,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="239" spans="1:26" ht="15">
+    <row r="239" spans="1:26" ht="15" hidden="1">
       <c r="A239" t="s">
         <v>1289</v>
       </c>
@@ -26090,7 +26075,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="240" spans="1:26" ht="15">
+    <row r="240" spans="1:26" ht="15" hidden="1">
       <c r="A240" t="s">
         <v>1296</v>
       </c>
@@ -26170,7 +26155,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="241" spans="1:26" ht="15">
+    <row r="241" spans="1:26" ht="15" hidden="1">
       <c r="A241" t="s">
         <v>1301</v>
       </c>
@@ -26250,7 +26235,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="242" spans="1:26" ht="15">
+    <row r="242" spans="1:26" ht="15" hidden="1">
       <c r="A242" s="1">
         <v>46059.458333333336</v>
       </c>
@@ -26330,7 +26315,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="243" spans="1:26" ht="15">
+    <row r="243" spans="1:26" ht="15" hidden="1">
       <c r="A243" s="1">
         <v>46059.636111111111</v>
       </c>
@@ -26410,7 +26395,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="244" spans="1:26" ht="15">
+    <row r="244" spans="1:26" ht="15" hidden="1">
       <c r="A244" t="s">
         <v>1314</v>
       </c>
@@ -26490,7 +26475,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="245" spans="1:26" ht="15">
+    <row r="245" spans="1:26" ht="15" hidden="1">
       <c r="A245" s="1">
         <v>46207.529861111114</v>
       </c>
@@ -26570,7 +26555,7 @@
         <v>297</v>
       </c>
     </row>
-    <row r="246" spans="1:26" ht="15">
+    <row r="246" spans="1:26" ht="15" hidden="1">
       <c r="A246" t="s">
         <v>1323</v>
       </c>
@@ -26650,7 +26635,7 @@
         <v>297</v>
       </c>
     </row>
-    <row r="247" spans="1:26" ht="15">
+    <row r="247" spans="1:26" ht="15" hidden="1">
       <c r="A247" t="s">
         <v>1329</v>
       </c>
@@ -26730,7 +26715,7 @@
         <v>297</v>
       </c>
     </row>
-    <row r="248" spans="1:26" ht="15">
+    <row r="248" spans="1:26" ht="15" hidden="1">
       <c r="A248" t="s">
         <v>1331</v>
       </c>
@@ -26810,7 +26795,7 @@
         <v>436</v>
       </c>
     </row>
-    <row r="249" spans="1:26" ht="15">
+    <row r="249" spans="1:26" ht="15" hidden="1">
       <c r="A249" s="1">
         <v>46207.619444444441</v>
       </c>
@@ -26890,7 +26875,7 @@
         <v>436</v>
       </c>
     </row>
-    <row r="250" spans="1:26" ht="15">
+    <row r="250" spans="1:26" ht="15" hidden="1">
       <c r="A250" s="1">
         <v>46269.692361111112</v>
       </c>
@@ -26970,7 +26955,7 @@
         <v>436</v>
       </c>
     </row>
-    <row r="251" spans="1:26" ht="15">
+    <row r="251" spans="1:26" ht="15" hidden="1">
       <c r="A251" t="s">
         <v>1347</v>
       </c>
@@ -27050,7 +27035,7 @@
         <v>436</v>
       </c>
     </row>
-    <row r="252" spans="1:26" ht="15">
+    <row r="252" spans="1:26" ht="15" hidden="1">
       <c r="A252" t="s">
         <v>1353</v>
       </c>
@@ -27130,7 +27115,7 @@
         <v>436</v>
       </c>
     </row>
-    <row r="253" spans="1:26" ht="15">
+    <row r="253" spans="1:26" ht="15" hidden="1">
       <c r="A253" t="s">
         <v>1359</v>
       </c>
@@ -27210,7 +27195,7 @@
         <v>436</v>
       </c>
     </row>
-    <row r="254" spans="1:26" ht="15">
+    <row r="254" spans="1:26" ht="15" hidden="1">
       <c r="A254" s="1">
         <v>46117.65347222222</v>
       </c>
@@ -27290,7 +27275,7 @@
         <v>436</v>
       </c>
     </row>
-    <row r="255" spans="1:26" ht="15">
+    <row r="255" spans="1:26" ht="15" hidden="1">
       <c r="A255" s="1">
         <v>46361.520138888889</v>
       </c>
@@ -27370,7 +27355,7 @@
         <v>436</v>
       </c>
     </row>
-    <row r="256" spans="1:26" ht="15">
+    <row r="256" spans="1:26" ht="15" hidden="1">
       <c r="A256" s="1">
         <v>46087.530555555553</v>
       </c>
@@ -27450,7 +27435,7 @@
         <v>436</v>
       </c>
     </row>
-    <row r="257" spans="1:26" ht="15">
+    <row r="257" spans="1:26" ht="15" hidden="1">
       <c r="A257" s="1">
         <v>46087.604861111111</v>
       </c>
@@ -27530,7 +27515,7 @@
         <v>436</v>
       </c>
     </row>
-    <row r="258" spans="1:26" ht="15">
+    <row r="258" spans="1:26" ht="15" hidden="1">
       <c r="A258" s="1">
         <v>46271.511805555558</v>
       </c>
@@ -27610,7 +27595,7 @@
         <v>436</v>
       </c>
     </row>
-    <row r="259" spans="1:26" ht="29.25">
+    <row r="259" spans="1:26" ht="29.25" hidden="1">
       <c r="A259" t="s">
         <v>1386</v>
       </c>
@@ -27690,7 +27675,7 @@
         <v>246</v>
       </c>
     </row>
-    <row r="260" spans="1:26" ht="15">
+    <row r="260" spans="1:26" ht="15" hidden="1">
       <c r="A260" t="s">
         <v>1392</v>
       </c>
@@ -27770,7 +27755,7 @@
         <v>436</v>
       </c>
     </row>
-    <row r="261" spans="1:26" ht="15">
+    <row r="261" spans="1:26" ht="15" hidden="1">
       <c r="A261" t="s">
         <v>1401</v>
       </c>
@@ -27850,7 +27835,7 @@
         <v>436</v>
       </c>
     </row>
-    <row r="262" spans="1:26" ht="15">
+    <row r="262" spans="1:26" ht="15" hidden="1">
       <c r="A262" t="s">
         <v>1407</v>
       </c>
@@ -27930,7 +27915,7 @@
         <v>436</v>
       </c>
     </row>
-    <row r="263" spans="1:26" ht="15">
+    <row r="263" spans="1:26" ht="15" hidden="1">
       <c r="A263" t="s">
         <v>1411</v>
       </c>
@@ -28090,7 +28075,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="265" spans="1:26" ht="15">
+    <row r="265" spans="1:26" ht="15" hidden="1">
       <c r="A265" t="s">
         <v>1426</v>
       </c>
@@ -28170,7 +28155,7 @@
         <v>225</v>
       </c>
     </row>
-    <row r="266" spans="1:26" ht="29.25">
+    <row r="266" spans="1:26" ht="29.25" hidden="1">
       <c r="A266" t="s">
         <v>1430</v>
       </c>
@@ -28250,7 +28235,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="267" spans="1:26" ht="15">
+    <row r="267" spans="1:26" ht="15" hidden="1">
       <c r="A267" t="s">
         <v>1437</v>
       </c>
@@ -28330,7 +28315,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="268" spans="1:26" ht="15">
+    <row r="268" spans="1:26" ht="15" hidden="1">
       <c r="A268" t="s">
         <v>1445</v>
       </c>
@@ -28410,7 +28395,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="269" spans="1:26" ht="15">
+    <row r="269" spans="1:26" ht="15" hidden="1">
       <c r="A269" t="s">
         <v>1450</v>
       </c>
@@ -28490,7 +28475,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="270" spans="1:26" ht="15">
+    <row r="270" spans="1:26" ht="15" hidden="1">
       <c r="A270" t="s">
         <v>1455</v>
       </c>
@@ -28570,7 +28555,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="271" spans="1:26" ht="15">
+    <row r="271" spans="1:26" ht="15" hidden="1">
       <c r="A271" s="1">
         <v>46147.468055555553</v>
       </c>
@@ -28650,7 +28635,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="272" spans="1:26" ht="15">
+    <row r="272" spans="1:26" ht="15" hidden="1">
       <c r="A272" s="1">
         <v>46147.661111111112</v>
       </c>
@@ -28730,7 +28715,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="273" spans="1:26" ht="15">
+    <row r="273" spans="1:26" ht="15" hidden="1">
       <c r="A273" s="1">
         <v>46147.756944444445</v>
       </c>
@@ -28810,7 +28795,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="274" spans="1:26" ht="15">
+    <row r="274" spans="1:26" ht="15" hidden="1">
       <c r="A274" s="1">
         <v>46208.526388888888</v>
       </c>
@@ -28890,7 +28875,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="275" spans="1:26" ht="15">
+    <row r="275" spans="1:26" ht="15" hidden="1">
       <c r="A275" s="1">
         <v>46208.52847222222</v>
       </c>
@@ -28970,7 +28955,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="276" spans="1:26" ht="15">
+    <row r="276" spans="1:26" ht="15" hidden="1">
       <c r="A276" s="1">
         <v>46331.429166666669</v>
       </c>
@@ -29050,7 +29035,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="277" spans="1:26" ht="15">
+    <row r="277" spans="1:26" ht="15" hidden="1">
       <c r="A277" t="s">
         <v>1489</v>
       </c>
@@ -29130,7 +29115,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="278" spans="1:26" ht="15">
+    <row r="278" spans="1:26" ht="15" hidden="1">
       <c r="A278" t="s">
         <v>1496</v>
       </c>
@@ -29210,7 +29195,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="279" spans="1:26" ht="15">
+    <row r="279" spans="1:26" ht="15" hidden="1">
       <c r="A279" t="s">
         <v>1500</v>
       </c>
@@ -29290,7 +29275,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="280" spans="1:26" ht="15">
+    <row r="280" spans="1:26" ht="15" hidden="1">
       <c r="A280" t="s">
         <v>1505</v>
       </c>
@@ -29370,7 +29355,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="281" spans="1:26" ht="15">
+    <row r="281" spans="1:26" ht="15" hidden="1">
       <c r="A281" s="1">
         <v>46059.638194444444</v>
       </c>
@@ -29450,7 +29435,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="282" spans="1:26" ht="15">
+    <row r="282" spans="1:26" ht="15" hidden="1">
       <c r="A282" s="1">
         <v>46301.695138888892</v>
       </c>
@@ -29530,7 +29515,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="283" spans="1:26" ht="15">
+    <row r="283" spans="1:26" ht="15" hidden="1">
       <c r="A283" s="1">
         <v>46332.383333333331</v>
       </c>
@@ -29610,7 +29595,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="284" spans="1:26" ht="15">
+    <row r="284" spans="1:26" ht="15" hidden="1">
       <c r="A284" t="s">
         <v>1526</v>
       </c>
@@ -29690,7 +29675,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="285" spans="1:26" ht="15">
+    <row r="285" spans="1:26" ht="15" hidden="1">
       <c r="A285" t="s">
         <v>1532</v>
       </c>
@@ -29770,7 +29755,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="286" spans="1:26" ht="15">
+    <row r="286" spans="1:26" ht="15" hidden="1">
       <c r="A286" t="s">
         <v>1537</v>
       </c>
@@ -29850,7 +29835,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="287" spans="1:26" ht="15">
+    <row r="287" spans="1:26" ht="15" hidden="1">
       <c r="A287" t="s">
         <v>1542</v>
       </c>
@@ -29930,7 +29915,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="288" spans="1:26" ht="15">
+    <row r="288" spans="1:26" ht="15" hidden="1">
       <c r="A288" t="s">
         <v>1546</v>
       </c>
@@ -30010,7 +29995,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="289" spans="1:26" ht="15">
+    <row r="289" spans="1:26" ht="15" hidden="1">
       <c r="A289" t="s">
         <v>1551</v>
       </c>
@@ -30090,7 +30075,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="290" spans="1:26" ht="15">
+    <row r="290" spans="1:26" ht="15" hidden="1">
       <c r="A290" t="s">
         <v>1556</v>
       </c>
@@ -30170,7 +30155,7 @@
         <v>1564</v>
       </c>
     </row>
-    <row r="291" spans="1:26" ht="15">
+    <row r="291" spans="1:26" ht="15" hidden="1">
       <c r="A291" s="1">
         <v>46087.504166666666</v>
       </c>
@@ -30250,7 +30235,7 @@
         <v>1564</v>
       </c>
     </row>
-    <row r="292" spans="1:26" ht="15">
+    <row r="292" spans="1:26" ht="15" hidden="1">
       <c r="A292" t="s">
         <v>1566</v>
       </c>
@@ -30330,7 +30315,7 @@
         <v>1564</v>
       </c>
     </row>
-    <row r="293" spans="1:26" ht="15">
+    <row r="293" spans="1:26" ht="15" hidden="1">
       <c r="A293" t="s">
         <v>1570</v>
       </c>
@@ -33370,7 +33355,7 @@
         <v>518</v>
       </c>
     </row>
-    <row r="331" spans="1:26" ht="15">
+    <row r="331" spans="1:26" ht="15" hidden="1">
       <c r="A331" t="s">
         <v>1696</v>
       </c>
@@ -33450,7 +33435,7 @@
         <v>297</v>
       </c>
     </row>
-    <row r="332" spans="1:26" ht="15">
+    <row r="332" spans="1:26" ht="15" hidden="1">
       <c r="A332" t="s">
         <v>1700</v>
       </c>
@@ -33530,7 +33515,7 @@
         <v>297</v>
       </c>
     </row>
-    <row r="333" spans="1:26" ht="15">
+    <row r="333" spans="1:26" ht="15" hidden="1">
       <c r="A333" t="s">
         <v>1706</v>
       </c>
@@ -33610,7 +33595,7 @@
         <v>297</v>
       </c>
     </row>
-    <row r="334" spans="1:26" ht="15">
+    <row r="334" spans="1:26" ht="15" hidden="1">
       <c r="A334" t="s">
         <v>1713</v>
       </c>
@@ -33690,7 +33675,7 @@
         <v>297</v>
       </c>
     </row>
-    <row r="335" spans="1:26" ht="15">
+    <row r="335" spans="1:26" ht="15" hidden="1">
       <c r="A335" t="s">
         <v>1718</v>
       </c>
@@ -33770,7 +33755,7 @@
         <v>297</v>
       </c>
     </row>
-    <row r="336" spans="1:26" ht="15">
+    <row r="336" spans="1:26" ht="15" hidden="1">
       <c r="A336" t="s">
         <v>1726</v>
       </c>
@@ -33850,7 +33835,7 @@
         <v>225</v>
       </c>
     </row>
-    <row r="337" spans="1:26" ht="15">
+    <row r="337" spans="1:26" ht="15" hidden="1">
       <c r="A337" s="1">
         <v>46059.597222222219</v>
       </c>
@@ -33930,7 +33915,7 @@
         <v>225</v>
       </c>
     </row>
-    <row r="338" spans="1:26" ht="15">
+    <row r="338" spans="1:26" ht="15" hidden="1">
       <c r="A338" s="1">
         <v>46271.50277777778</v>
       </c>
@@ -34010,7 +33995,7 @@
         <v>225</v>
       </c>
     </row>
-    <row r="339" spans="1:26" ht="15">
+    <row r="339" spans="1:26" ht="15" hidden="1">
       <c r="A339" s="1">
         <v>46026.671527777777</v>
       </c>
@@ -34090,7 +34075,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="340" spans="1:26" ht="15">
+    <row r="340" spans="1:26" ht="15" hidden="1">
       <c r="A340" t="s">
         <v>1744</v>
       </c>
@@ -34170,7 +34155,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="341" spans="1:26" ht="15">
+    <row r="341" spans="1:26" ht="15" hidden="1">
       <c r="A341" t="s">
         <v>1749</v>
       </c>
@@ -34250,7 +34235,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="342" spans="1:26" ht="15">
+    <row r="342" spans="1:26" ht="15" hidden="1">
       <c r="A342" t="s">
         <v>1755</v>
       </c>
@@ -34330,7 +34315,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="343" spans="1:26" ht="43.5">
+    <row r="343" spans="1:26" ht="43.5" hidden="1">
       <c r="A343" t="s">
         <v>1760</v>
       </c>
@@ -34410,7 +34395,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="344" spans="1:26" ht="43.5">
+    <row r="344" spans="1:26" ht="43.5" hidden="1">
       <c r="A344" t="s">
         <v>1765</v>
       </c>
@@ -34490,7 +34475,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="345" spans="1:26" ht="43.5">
+    <row r="345" spans="1:26" ht="43.5" hidden="1">
       <c r="A345" t="s">
         <v>1769</v>
       </c>
@@ -34570,7 +34555,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="346" spans="1:26" ht="43.5">
+    <row r="346" spans="1:26" ht="43.5" hidden="1">
       <c r="A346" t="s">
         <v>1773</v>
       </c>
@@ -34650,7 +34635,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="347" spans="1:26" ht="15">
+    <row r="347" spans="1:26" ht="15" hidden="1">
       <c r="A347" t="s">
         <v>1777</v>
       </c>
@@ -34730,7 +34715,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="348" spans="1:26" ht="15">
+    <row r="348" spans="1:26" ht="15" hidden="1">
       <c r="A348" t="s">
         <v>1782</v>
       </c>
@@ -34810,7 +34795,7 @@
         <v>297</v>
       </c>
     </row>
-    <row r="349" spans="1:26" ht="15">
+    <row r="349" spans="1:26" ht="15" hidden="1">
       <c r="A349" t="s">
         <v>1785</v>
       </c>
@@ -34890,7 +34875,7 @@
         <v>246</v>
       </c>
     </row>
-    <row r="350" spans="1:26" ht="15">
+    <row r="350" spans="1:26" ht="15" hidden="1">
       <c r="A350" s="1">
         <v>46238.672222222223</v>
       </c>
@@ -34970,7 +34955,7 @@
         <v>297</v>
       </c>
     </row>
-    <row r="351" spans="1:26" ht="15">
+    <row r="351" spans="1:26" ht="15" hidden="1">
       <c r="A351" s="1">
         <v>46148.45</v>
       </c>
@@ -35050,7 +35035,7 @@
         <v>297</v>
       </c>
     </row>
-    <row r="352" spans="1:26" ht="15">
+    <row r="352" spans="1:26" ht="15" hidden="1">
       <c r="A352" t="s">
         <v>1797</v>
       </c>
@@ -35130,7 +35115,7 @@
         <v>436</v>
       </c>
     </row>
-    <row r="353" spans="1:26" ht="15">
+    <row r="353" spans="1:26" ht="15" hidden="1">
       <c r="A353" t="s">
         <v>1806</v>
       </c>
@@ -35210,7 +35195,7 @@
         <v>436</v>
       </c>
     </row>
-    <row r="354" spans="1:26" ht="15">
+    <row r="354" spans="1:26" ht="15" hidden="1">
       <c r="A354" t="s">
         <v>1810</v>
       </c>
@@ -35290,7 +35275,7 @@
         <v>436</v>
       </c>
     </row>
-    <row r="355" spans="1:26" ht="15">
+    <row r="355" spans="1:26" ht="15" hidden="1">
       <c r="A355" t="s">
         <v>1816</v>
       </c>
@@ -35370,7 +35355,7 @@
         <v>436</v>
       </c>
     </row>
-    <row r="356" spans="1:26" ht="15">
+    <row r="356" spans="1:26" ht="15" hidden="1">
       <c r="A356" t="s">
         <v>1822</v>
       </c>
@@ -35450,7 +35435,7 @@
         <v>436</v>
       </c>
     </row>
-    <row r="357" spans="1:26" ht="15">
+    <row r="357" spans="1:26" ht="15" hidden="1">
       <c r="A357" s="1">
         <v>46117.449305555558</v>
       </c>
@@ -35530,7 +35515,7 @@
         <v>436</v>
       </c>
     </row>
-    <row r="358" spans="1:26" ht="15">
+    <row r="358" spans="1:26" ht="15" hidden="1">
       <c r="A358" s="1">
         <v>46117.450694444444</v>
       </c>
@@ -35610,7 +35595,7 @@
         <v>436</v>
       </c>
     </row>
-    <row r="359" spans="1:26" ht="15">
+    <row r="359" spans="1:26" ht="15" hidden="1">
       <c r="A359" s="1">
         <v>46178.648611111108</v>
       </c>
@@ -35690,7 +35675,7 @@
         <v>436</v>
       </c>
     </row>
-    <row r="360" spans="1:26" ht="15">
+    <row r="360" spans="1:26" ht="15" hidden="1">
       <c r="A360" s="1">
         <v>46239.490972222222</v>
       </c>
@@ -35770,7 +35755,7 @@
         <v>436</v>
       </c>
     </row>
-    <row r="361" spans="1:26" ht="15">
+    <row r="361" spans="1:26" ht="15" hidden="1">
       <c r="A361" t="s">
         <v>1841</v>
       </c>
@@ -35850,7 +35835,7 @@
         <v>436</v>
       </c>
     </row>
-    <row r="362" spans="1:26" ht="15">
+    <row r="362" spans="1:26" ht="15" hidden="1">
       <c r="A362" t="s">
         <v>1846</v>
       </c>
@@ -35930,7 +35915,7 @@
         <v>436</v>
       </c>
     </row>
-    <row r="363" spans="1:26" ht="15">
+    <row r="363" spans="1:26" ht="15" hidden="1">
       <c r="A363" s="1">
         <v>46207.51666666667</v>
       </c>
@@ -36010,7 +35995,7 @@
         <v>436</v>
       </c>
     </row>
-    <row r="364" spans="1:26" ht="15">
+    <row r="364" spans="1:26" ht="15" hidden="1">
       <c r="A364" s="1">
         <v>46269.529861111114</v>
       </c>
@@ -36090,7 +36075,7 @@
         <v>436</v>
       </c>
     </row>
-    <row r="365" spans="1:26" ht="15">
+    <row r="365" spans="1:26" ht="15" hidden="1">
       <c r="A365" t="s">
         <v>1861</v>
       </c>
@@ -36170,7 +36155,7 @@
         <v>436</v>
       </c>
     </row>
-    <row r="366" spans="1:26" ht="15">
+    <row r="366" spans="1:26" ht="15" hidden="1">
       <c r="A366" t="s">
         <v>1865</v>
       </c>
@@ -36250,7 +36235,7 @@
         <v>436</v>
       </c>
     </row>
-    <row r="367" spans="1:26" ht="15">
+    <row r="367" spans="1:26" ht="15" hidden="1">
       <c r="A367" t="s">
         <v>1869</v>
       </c>
@@ -36330,7 +36315,7 @@
         <v>436</v>
       </c>
     </row>
-    <row r="368" spans="1:26" ht="15">
+    <row r="368" spans="1:26" ht="15" hidden="1">
       <c r="A368" s="1">
         <v>46118.513888888891</v>
       </c>

</xml_diff>

<commit_message>
Update :- Vtiger Integration and Quota Template Implementation
</commit_message>
<xml_diff>
--- a/files/Opportunity Pipeline Q1.xlsx
+++ b/files/Opportunity Pipeline Q1.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Opportunity Pipeline Q1" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Opportunity Pipeline Q1" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>

</xml_diff>